<commit_message>
Record production Baseline run on Mesh 4; unlock PEC for Run 1 (1.433)
</commit_message>
<xml_diff>
--- a/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
+++ b/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
@@ -4391,18 +4391,42 @@
           <t>Baseline</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="9" t="n"/>
-      <c r="I2" s="9" t="n"/>
-      <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
-      <c r="L2" s="9" t="n"/>
-      <c r="M2" s="9" t="n"/>
+      <c r="B2" s="9" t="n">
+        <v>0.41748124</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>0.41747989</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>10.590583</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>519.09171</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>660.03433</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>0.07788985</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>35607.497</v>
+      </c>
+      <c r="K2" s="9" t="n">
+        <v>16106.493</v>
+      </c>
+      <c r="L2" s="9" t="n">
+        <v>0.07295852799999999</v>
+      </c>
+      <c r="M2" s="9" t="n">
+        <v>0.61857802</v>
+      </c>
       <c r="N2" s="9" t="n"/>
       <c r="O2" s="9" t="n"/>
       <c r="P2" s="9" t="n"/>

</xml_diff>

<commit_message>
Log Run 8 fluid properties (Fe2O3-GO, phi=2%)
</commit_message>
<xml_diff>
--- a/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
+++ b/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
@@ -3467,41 +3467,32 @@
       <c r="A10" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="5">
-        <f>'Run Matrix (Inputs)'!$H$10/100/2</f>
-        <v/>
-      </c>
-      <c r="C10" s="5">
-        <f>IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$10,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$10,Constants!$A$29:$A$34,0)),""))</f>
-        <v/>
-      </c>
-      <c r="D10" s="5">
-        <f>IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$10,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$10,Constants!$A$29:$A$34,0)),""))</f>
-        <v/>
-      </c>
-      <c r="E10" s="5">
-        <f>IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$10,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$10,Constants!$A$29:$A$34,0)),""))</f>
-        <v/>
-      </c>
-      <c r="F10" s="5">
-        <f>IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$10,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$10,Constants!$A$29:$A$34,0)),""))</f>
-        <v/>
-      </c>
-      <c r="G10" s="5">
-        <f>IF(OR($C$10="",$E$10=""),"",(1-'Run Matrix (Inputs)'!$H$10/100)*Constants!$C$22+$B$10*$C$10+$B$10*$E$10)</f>
-        <v/>
-      </c>
-      <c r="H10" s="5">
-        <f>IF(OR(OR($C$10="",$E$10=""),$G$10=""),"",((1-'Run Matrix (Inputs)'!$H$10/100)*Constants!$C$22*Constants!$C$23+$B$10*$C$10*$D$10+$B$10*$E$10*$F$10)/$G$10)</f>
-        <v/>
-      </c>
-      <c r="I10" s="5">
-        <f>Constants!$C$24*(1+Constants!$C$16*'Run Matrix (Inputs)'!$H$10/100)</f>
-        <v/>
-      </c>
-      <c r="J10" s="5">
-        <f>Constants!$C$25*((1+Constants!$C$17*$B$10+Constants!$C$18*$B$10^2)+(1+Constants!$C$17*$B$10+Constants!$C$18*$B$10^2))</f>
-        <v/>
+      <c r="B10" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>5180</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>670</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>717</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>802.056</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>1850.617</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>0.102577</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>0.0017911</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="6">

</xml_diff>

<commit_message>
Log Run 6 results: PEC~1.0, larger promoter drives friction up more than Nu
</commit_message>
<xml_diff>
--- a/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
+++ b/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
@@ -2868,11 +2868,26 @@
       <c r="A8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
+      <c r="B8" s="9" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>5032279</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>1869731</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>0.84882</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0.010296</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Min Orthogonal Quality right at the 0.01 edge (barely clears) - watch item for larger-promoter runs.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="6">
       <c r="A9" s="5" t="n">
@@ -4550,18 +4565,42 @@
       <c r="A8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
-      <c r="L8" s="9" t="n"/>
-      <c r="M8" s="9" t="n"/>
+      <c r="B8" s="9" t="n">
+        <v>0.81956674</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>0.81953926</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>212.57862</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>500</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>510.15269</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>618.8718699999999</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>0.7149851699999999</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>35610.415</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>15659.348</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>0.046114454</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>0.49609798</v>
+      </c>
       <c r="N8" s="9" t="n"/>
       <c r="O8" s="9" t="n"/>
       <c r="P8" s="9" t="n"/>

</xml_diff>

<commit_message>
Mark Run 8 as invalid (mesh quality failure) in master workbook, red-highlighted
</commit_message>
<xml_diff>
--- a/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
+++ b/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
@@ -61,7 +61,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +72,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF9C4"/>
         <bgColor rgb="FFFFFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,7 +99,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -123,6 +128,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1627,56 +1636,56 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="6">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="10" t="n">
         <v>3.03</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="10" t="n">
         <v>0.53</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="10" t="n">
         <v>0.08</v>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Fe2O3-GO</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Fe2O3</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>GO</t>
         </is>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="10" t="n">
         <v>200</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="K10" s="10" t="n">
         <v>2.8</v>
       </c>
-      <c r="L10" s="5" t="n">
+      <c r="L10" s="10" t="n">
         <v>29.4</v>
       </c>
-      <c r="M10" s="5" t="n">
+      <c r="M10" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="10">
         <f>Constants!$C$7</f>
         <v/>
       </c>
-      <c r="O10" s="5">
+      <c r="O10" s="10">
         <f>Constants!$C$8</f>
         <v/>
       </c>
@@ -2883,7 +2892,7 @@
       <c r="F8" s="9" t="n">
         <v>0.010296</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Min Orthogonal Quality right at the 0.01 edge (barely clears) - watch item for larger-promoter runs.</t>
         </is>
@@ -2900,14 +2909,29 @@
       <c r="F9" s="9" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="6">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
+      <c r="B10" s="10" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>6293136</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>2404391</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>0.84882</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>0.009691399999999999</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>INVALID - Min Orthogonal Quality 0.0096914 below 0.01 threshold (Max Aspect Ratio 959.99, near ANSYS failure limit 1000). Solution diverged. Needs finer local mesh in tight annulus region (dpo=35mm, tightest gap of any run tested) before re-running.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="6">
       <c r="A11" s="5" t="n">
@@ -3479,34 +3503,34 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="6">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="10" t="n">
         <v>0.01</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="10" t="n">
         <v>5180</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="10" t="n">
         <v>670</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="10" t="n">
         <v>1800</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="10" t="n">
         <v>717</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="10" t="n">
         <v>802.056</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="10" t="n">
         <v>1850.617</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="10" t="n">
         <v>0.102577</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="10" t="n">
         <v>0.0017911</v>
       </c>
     </row>
@@ -4626,24 +4650,24 @@
       <c r="P9" s="9" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="6">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n"/>
-      <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
-      <c r="M10" s="9" t="n"/>
-      <c r="N10" s="9" t="n"/>
-      <c r="O10" s="9" t="n"/>
-      <c r="P10" s="9" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="10" t="n"/>
+      <c r="J10" s="10" t="n"/>
+      <c r="K10" s="10" t="n"/>
+      <c r="L10" s="10" t="n"/>
+      <c r="M10" s="10" t="n"/>
+      <c r="N10" s="10" t="n"/>
+      <c r="O10" s="10" t="n"/>
+      <c r="P10" s="10" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="6">
       <c r="A11" s="5" t="n">
@@ -5689,70 +5713,70 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="6">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="10">
         <f>(PI()*Constants!$C$4^2/4-('Run Matrix (Inputs)'!$J$10/1000)^2)+('Run Matrix (Inputs)'!$L$10/1000)^2</f>
         <v/>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="10">
         <f>IFERROR('Fluent Raw Results'!$B$10/('Fluid Properties'!$G$10*$B$10),"")</f>
         <v/>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="10">
         <f>IFERROR('Fluid Properties'!$G$10*$C$10*Constants!$C$4/'Fluid Properties'!$J$10,"")</f>
         <v/>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="10">
         <f>IF(OR('Fluent Raw Results'!$F$10="",'Fluent Raw Results'!$G$10=""),"",('Fluent Raw Results'!$F$10+'Fluent Raw Results'!$G$10)/2)</f>
         <v/>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="10">
         <f>IF(OR('Fluent Raw Results'!$D$10="",'Fluent Raw Results'!$E$10=""),"",'Fluent Raw Results'!$D$10-'Fluent Raw Results'!$E$10)</f>
         <v/>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="10">
         <f>IFERROR(2*'Fluent Raw Results'!$I$10/('Fluid Properties'!$G$10*$C$10^2),"")</f>
         <v/>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="10">
         <f>IFERROR('Fluent Raw Results'!$J$10/('Fluent Raw Results'!$H$10-$E$10),"")</f>
         <v/>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="10">
         <f>IFERROR($H$10*Constants!$C$4/'Fluid Properties'!$I$10,"")</f>
         <v/>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="10">
         <f>IFERROR('Fluent Raw Results'!$B$10*'Fluid Properties'!$H$10*('Fluent Raw Results'!$G$10-'Fluent Raw Results'!$F$10),"")</f>
         <v/>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="10">
         <f>IFERROR(('Fluent Raw Results'!$B$10/'Fluid Properties'!$G$10)*$F$10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="10">
         <f>IFERROR(($J$10-$K$10/Constants!$C$13)/(Constants!$C$9*Constants!$C$10),"")</f>
         <v/>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="10">
         <f>IFERROR('Fluent Raw Results'!$B$10*'Fluid Properties'!$H$10*(('Fluent Raw Results'!$G$10-'Fluent Raw Results'!$F$10)-Constants!$C$11*LN('Fluent Raw Results'!$G$10/'Fluent Raw Results'!$F$10))/(Constants!$C$9*Constants!$C$10*(1+(1/3)*(Constants!$C$11/Constants!$C$12)^4-(4/3)*(Constants!$C$11/Constants!$C$12))),"")</f>
         <v/>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="10">
         <f>IFERROR(($I$10/$I$2)/($G$10/$G$2)^(1/3),"")</f>
         <v/>
       </c>
-      <c r="O10" s="5">
+      <c r="O10" s="10">
         <f>IFERROR('Fluent Raw Results'!$O$10/'Fluent Raw Results'!$N$10,"")</f>
         <v/>
       </c>
-      <c r="P10" s="5">
+      <c r="P10" s="10">
         <f>IFERROR('Fluent Raw Results'!$N$10/'Fluent Raw Results'!$N$2,"")</f>
         <v/>
       </c>
-      <c r="Q10" s="5">
+      <c r="Q10" s="10">
         <f>IFERROR(ABS('Fluent Raw Results'!$B$10-'Fluent Raw Results'!$C$10)/'Fluent Raw Results'!$B$10*100,"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Log Run 12 results: PEC=0.952, longer twist pitch + thicker wall drags PEC below Run 1/6
</commit_message>
<xml_diff>
--- a/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
+++ b/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="159">
   <si>
     <t xml:space="preserve">PTSC 27-Run Master Results Workbook</t>
   </si>
@@ -377,6 +377,9 @@
   </si>
   <si>
     <t xml:space="preserve">INVALID - Min Orthogonal Quality 0.0096914 below 0.01 threshold (Max Aspect Ratio 959.99, near ANSYS failure limit 1000). Solution diverged. Needs finer local mesh in tight annulus region (dpo=35mm, tightest gap of any run tested) before re-running.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean mesh, well above 0.01 quality target.</t>
   </si>
   <si>
     <t xml:space="preserve">phi1 (=phi2, even-split assumption)</t>
@@ -601,7 +604,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -623,10 +626,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3009,7 +3008,7 @@
       <c r="F10" s="5" t="n">
         <v>0.0096914</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="5" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3047,11 +3046,24 @@
       <c r="A14" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
+      <c r="B14" s="4" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>4378599</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1625862</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0.84954</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0.016175</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
@@ -3234,31 +3246,31 @@
         <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4402,49 +4414,49 @@
         <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4763,18 +4775,42 @@
       <c r="A14" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
+      <c r="B14" s="4" t="n">
+        <v>0.85199436</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>0.85202275</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>128.01882</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>509.55327</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>636.55458</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.55386734</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>35606.134</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>15656.949</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>0.040340282</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0.49711385</v>
+      </c>
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
@@ -5107,52 +5143,52 @@
         <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5208,14 +5244,14 @@
         <v>0.176177681878176</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="O2" s="1" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$O$2/'Fluent Raw Results'!$N$2,"")</f>
         <v/>
       </c>
       <c r="P2" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Q2" s="1" t="n">
         <f aca="false">IFERROR(ABS('Fluent Raw Results'!$B$2-'Fluent Raw Results'!$C$2)/'Fluent Raw Results'!$B$2*100,"")</f>
@@ -5991,51 +6027,51 @@
       </c>
       <c r="C14" s="1" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$14/('Fluid Properties'!$G$14*$B$14),"")</f>
-        <v>0</v>
+        <v>0.336634590890097</v>
       </c>
       <c r="D14" s="1" t="n">
         <f aca="false">IFERROR('Fluid Properties'!$G$14*$C$14*Constants!$C$4/'Fluid Properties'!$J$14,"")</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="1" t="str">
+        <v>9986.1785306904</v>
+      </c>
+      <c r="E14" s="1" t="n">
         <f aca="false">IF(OR('Fluent Raw Results'!$F$14="",'Fluent Raw Results'!$G$14=""),"",('Fluent Raw Results'!$F$14+'Fluent Raw Results'!$G$14)/2)</f>
-        <v/>
-      </c>
-      <c r="F14" s="1" t="str">
+        <v>504.776635</v>
+      </c>
+      <c r="F14" s="1" t="n">
         <f aca="false">IF(OR('Fluent Raw Results'!$D$14="",'Fluent Raw Results'!$E$14=""),"",'Fluent Raw Results'!$D$14-'Fluent Raw Results'!$E$14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="1" t="str">
+        <v>128.01882</v>
+      </c>
+      <c r="G14" s="1" t="n">
         <f aca="false">IFERROR(2*'Fluent Raw Results'!$I$14/('Fluid Properties'!$G$14*$C$14^2),"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="1" t="str">
+        <v>0.0128464371942182</v>
+      </c>
+      <c r="H14" s="1" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$J$14/('Fluent Raw Results'!$H$14-$E$14),"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="1" t="str">
+        <v>270.197975844896</v>
+      </c>
+      <c r="I14" s="1" t="n">
         <f aca="false">IFERROR($H$14*Constants!$C$4/'Fluid Properties'!$I$14,"")</f>
-        <v/>
+        <v>182.49280483134</v>
       </c>
       <c r="J14" s="1" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$14*'Fluid Properties'!$H$14*('Fluent Raw Results'!$G$14-'Fluent Raw Results'!$F$14),"")</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="1" t="str">
+        <v>15730.4688087533</v>
+      </c>
+      <c r="K14" s="1" t="n">
         <f aca="false">IFERROR(('Fluent Raw Results'!$B$14/'Fluid Properties'!$G$14)*$F$14,"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="1" t="str">
+        <v>0.143342496804968</v>
+      </c>
+      <c r="L14" s="1" t="n">
         <f aca="false">IFERROR(($J$14-$K$14/Constants!$C$13)/(Constants!$C$9*Constants!$C$10),"")</f>
-        <v/>
-      </c>
-      <c r="M14" s="1" t="str">
+        <v>0.40127528062323</v>
+      </c>
+      <c r="M14" s="1" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$14*'Fluid Properties'!$H$14*(('Fluent Raw Results'!$G$14-'Fluent Raw Results'!$F$14)-Constants!$C$11*LN('Fluent Raw Results'!$G$14/'Fluent Raw Results'!$F$14))/(Constants!$C$9*Constants!$C$10*(1+(1/3)*(Constants!$C$11/Constants!$C$12)^4-(4/3)*(Constants!$C$11/Constants!$C$12))),"")</f>
-        <v/>
-      </c>
-      <c r="N14" s="1" t="str">
+        <v>0.174844061060482</v>
+      </c>
+      <c r="N14" s="1" t="n">
         <f aca="false">IFERROR(($I$14/$I$2)/($G$14/$G$2)^(1/3),"")</f>
-        <v/>
+        <v>0.951632344021105</v>
       </c>
       <c r="O14" s="1" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$O$14/'Fluent Raw Results'!$N$14,"")</f>
@@ -6045,9 +6081,9 @@
         <f aca="false">IFERROR('Fluent Raw Results'!$N$14/'Fluent Raw Results'!$N$2,"")</f>
         <v/>
       </c>
-      <c r="Q14" s="1" t="str">
+      <c r="Q14" s="1" t="n">
         <f aca="false">IFERROR(ABS('Fluent Raw Results'!$B$14-'Fluent Raw Results'!$C$14)/'Fluent Raw Results'!$B$14*100,"")</f>
-        <v/>
+        <v>0.00333218168252901</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Pre-log fluid properties for remaining Fe2O3-GO runs (14,16,20,22,27)
</commit_message>
<xml_diff>
--- a/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
+++ b/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
@@ -3817,40 +3817,31 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="n">
-        <f aca="false">'Run Matrix (Inputs)'!$H$16/100/2</f>
         <v>0.005</v>
       </c>
       <c r="C16" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$16,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$16,Constants!$A$29:$A$34,0)),""))</f>
         <v>5180</v>
       </c>
       <c r="D16" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$16,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$16,Constants!$A$29:$A$34,0)),""))</f>
         <v>670</v>
       </c>
       <c r="E16" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$16,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$16,Constants!$A$29:$A$34,0)),""))</f>
         <v>1800</v>
       </c>
       <c r="F16" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$16,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$16,Constants!$A$29:$A$34,0)),""))</f>
         <v>717</v>
       </c>
       <c r="G16" s="1" t="n">
-        <f aca="false">IF(OR($C$16="",$E$16=""),"",(1-'Run Matrix (Inputs)'!$H$16/100)*Constants!$C$22+$B$16*$C$16+$B$16*$E$16)</f>
         <v>774.628</v>
       </c>
       <c r="H16" s="1" t="n">
-        <f aca="false">IF(OR(OR($C$16="",$E$16=""),$G$16=""),"",((1-'Run Matrix (Inputs)'!$H$16/100)*Constants!$C$22*Constants!$C$23+$B$16*$C$16*$D$16+$B$16*$E$16*$F$16)/$G$16)</f>
-        <v>1904.33645052851</v>
+        <v>1904.34</v>
       </c>
       <c r="I16" s="1" t="n">
-        <f aca="false">Constants!$C$24*(1+Constants!$C$16*'Run Matrix (Inputs)'!$H$16/100)</f>
-        <v>0.09933857</v>
+        <v>0.09934</v>
       </c>
       <c r="J16" s="1" t="n">
-        <f aca="false">Constants!$C$25*((1+Constants!$C$17*$B$16+Constants!$C$18*$B$16^2)+(1+Constants!$C$17*$B$16+Constants!$C$18*$B$16^2))</f>
-        <v>0.0017157588</v>
+        <v>0.0017158</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3899,40 +3890,31 @@
         <v>16</v>
       </c>
       <c r="B18" s="1" t="n">
-        <f aca="false">'Run Matrix (Inputs)'!$H$18/100/2</f>
         <v>0.01</v>
       </c>
       <c r="C18" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$18,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$18,Constants!$A$29:$A$34,0)),""))</f>
         <v>5180</v>
       </c>
       <c r="D18" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$18,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$18,Constants!$A$29:$A$34,0)),""))</f>
         <v>670</v>
       </c>
       <c r="E18" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$18,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$18,Constants!$A$29:$A$34,0)),""))</f>
         <v>1800</v>
       </c>
       <c r="F18" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$18,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$18,Constants!$A$29:$A$34,0)),""))</f>
         <v>717</v>
       </c>
       <c r="G18" s="1" t="n">
-        <f aca="false">IF(OR($C$18="",$E$18=""),"",(1-'Run Matrix (Inputs)'!$H$18/100)*Constants!$C$22+$B$18*$C$18+$B$18*$E$18)</f>
         <v>802.056</v>
       </c>
       <c r="H18" s="1" t="n">
-        <f aca="false">IF(OR(OR($C$18="",$E$18=""),$G$18=""),"",((1-'Run Matrix (Inputs)'!$H$18/100)*Constants!$C$22*Constants!$C$23+$B$18*$C$18*$D$18+$B$18*$E$18*$F$18)/$G$18)</f>
-        <v>1850.6167549398</v>
+        <v>1850.62</v>
       </c>
       <c r="I18" s="1" t="n">
-        <f aca="false">Constants!$C$24*(1+Constants!$C$16*'Run Matrix (Inputs)'!$H$18/100)</f>
-        <v>0.10257714</v>
+        <v>0.102577</v>
       </c>
       <c r="J18" s="1" t="n">
-        <f aca="false">Constants!$C$25*((1+Constants!$C$17*$B$18+Constants!$C$18*$B$18^2)+(1+Constants!$C$17*$B$18+Constants!$C$18*$B$18^2))</f>
-        <v>0.0017911152</v>
+        <v>0.0017911</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4063,40 +4045,31 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="n">
-        <f aca="false">'Run Matrix (Inputs)'!$H$22/100/2</f>
         <v>0.0025</v>
       </c>
       <c r="C22" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$22,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$22,Constants!$A$29:$A$34,0)),""))</f>
         <v>5180</v>
       </c>
       <c r="D22" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$22,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$22,Constants!$A$29:$A$34,0)),""))</f>
         <v>670</v>
       </c>
       <c r="E22" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$22,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$22,Constants!$A$29:$A$34,0)),""))</f>
         <v>1800</v>
       </c>
       <c r="F22" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$22,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$22,Constants!$A$29:$A$34,0)),""))</f>
         <v>717</v>
       </c>
       <c r="G22" s="1" t="n">
-        <f aca="false">IF(OR($C$22="",$E$22=""),"",(1-'Run Matrix (Inputs)'!$H$22/100)*Constants!$C$22+$B$22*$C$22+$B$22*$E$22)</f>
         <v>760.914</v>
       </c>
       <c r="H22" s="1" t="n">
-        <f aca="false">IF(OR(OR($C$22="",$E$22=""),$G$22=""),"",((1-'Run Matrix (Inputs)'!$H$22/100)*Constants!$C$22*Constants!$C$23+$B$22*$C$22*$D$22+$B$22*$E$22*$F$22)/$G$22)</f>
-        <v>1932.64858840815</v>
+        <v>1932.65</v>
       </c>
       <c r="I22" s="1" t="n">
-        <f aca="false">Constants!$C$24*(1+Constants!$C$16*'Run Matrix (Inputs)'!$H$22/100)</f>
-        <v>0.097719285</v>
+        <v>0.09772</v>
       </c>
       <c r="J22" s="1" t="n">
-        <f aca="false">Constants!$C$25*((1+Constants!$C$17*$B$22+Constants!$C$18*$B$22^2)+(1+Constants!$C$17*$B$22+Constants!$C$18*$B$22^2))</f>
-        <v>0.0016929297</v>
+        <v>0.0016929</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4145,40 +4118,31 @@
         <v>22</v>
       </c>
       <c r="B24" s="1" t="n">
-        <f aca="false">'Run Matrix (Inputs)'!$H$24/100/2</f>
         <v>0.005</v>
       </c>
       <c r="C24" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$24,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$24,Constants!$A$29:$A$34,0)),""))</f>
         <v>5180</v>
       </c>
       <c r="D24" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$24,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$24,Constants!$A$29:$A$34,0)),""))</f>
         <v>670</v>
       </c>
       <c r="E24" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$24,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$24,Constants!$A$29:$A$34,0)),""))</f>
         <v>1800</v>
       </c>
       <c r="F24" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$24,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$24,Constants!$A$29:$A$34,0)),""))</f>
         <v>717</v>
       </c>
       <c r="G24" s="1" t="n">
-        <f aca="false">IF(OR($C$24="",$E$24=""),"",(1-'Run Matrix (Inputs)'!$H$24/100)*Constants!$C$22+$B$24*$C$24+$B$24*$E$24)</f>
         <v>774.628</v>
       </c>
       <c r="H24" s="1" t="n">
-        <f aca="false">IF(OR(OR($C$24="",$E$24=""),$G$24=""),"",((1-'Run Matrix (Inputs)'!$H$24/100)*Constants!$C$22*Constants!$C$23+$B$24*$C$24*$D$24+$B$24*$E$24*$F$24)/$G$24)</f>
-        <v>1904.33645052851</v>
+        <v>1904.34</v>
       </c>
       <c r="I24" s="1" t="n">
-        <f aca="false">Constants!$C$24*(1+Constants!$C$16*'Run Matrix (Inputs)'!$H$24/100)</f>
-        <v>0.09933857</v>
+        <v>0.09934</v>
       </c>
       <c r="J24" s="1" t="n">
-        <f aca="false">Constants!$C$25*((1+Constants!$C$17*$B$24+Constants!$C$18*$B$24^2)+(1+Constants!$C$17*$B$24+Constants!$C$18*$B$24^2))</f>
-        <v>0.0017157588</v>
+        <v>0.0017158</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4350,40 +4314,31 @@
         <v>27</v>
       </c>
       <c r="B29" s="1" t="n">
-        <f aca="false">'Run Matrix (Inputs)'!$H$29/100/2</f>
         <v>0.01</v>
       </c>
       <c r="C29" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$29,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$F$29,Constants!$A$29:$A$34,0)),""))</f>
         <v>5180</v>
       </c>
       <c r="D29" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$29,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$F$29,Constants!$A$29:$A$34,0)),""))</f>
         <v>670</v>
       </c>
       <c r="E29" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$29,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$B$29:$B$34,MATCH('Run Matrix (Inputs)'!$G$29,Constants!$A$29:$A$34,0)),""))</f>
         <v>1800</v>
       </c>
       <c r="F29" s="1" t="n">
-        <f aca="false">IF(IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$29,Constants!$A$29:$A$34,0)),"")="","",IFERROR(INDEX(Constants!$C$29:$C$34,MATCH('Run Matrix (Inputs)'!$G$29,Constants!$A$29:$A$34,0)),""))</f>
         <v>717</v>
       </c>
       <c r="G29" s="1" t="n">
-        <f aca="false">IF(OR($C$29="",$E$29=""),"",(1-'Run Matrix (Inputs)'!$H$29/100)*Constants!$C$22+$B$29*$C$29+$B$29*$E$29)</f>
         <v>802.056</v>
       </c>
       <c r="H29" s="1" t="n">
-        <f aca="false">IF(OR(OR($C$29="",$E$29=""),$G$29=""),"",((1-'Run Matrix (Inputs)'!$H$29/100)*Constants!$C$22*Constants!$C$23+$B$29*$C$29*$D$29+$B$29*$E$29*$F$29)/$G$29)</f>
-        <v>1850.6167549398</v>
+        <v>1850.62</v>
       </c>
       <c r="I29" s="1" t="n">
-        <f aca="false">Constants!$C$24*(1+Constants!$C$16*'Run Matrix (Inputs)'!$H$29/100)</f>
-        <v>0.10257714</v>
+        <v>0.102577</v>
       </c>
       <c r="J29" s="1" t="n">
-        <f aca="false">Constants!$C$25*((1+Constants!$C$17*$B$29+Constants!$C$18*$B$29^2)+(1+Constants!$C$17*$B$29+Constants!$C$18*$B$29^2))</f>
-        <v>0.0017911152</v>
+        <v>0.0017911</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark Run 16 as invalid (same dpo=35mm mesh quality failure as Run 8) - confirmed pattern
</commit_message>
<xml_diff>
--- a/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
+++ b/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="160">
   <si>
     <t xml:space="preserve">PTSC 27-Run Master Results Workbook</t>
   </si>
@@ -380,6 +380,9 @@
   </si>
   <si>
     <t xml:space="preserve">Clean mesh, well above 0.01 quality target.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVALID - same failure as Run 8: Min Orthogonal Quality 0.0092812, below 0.01 threshold. Solution diverged (T_wall=4925K, p_in~2.7e35). CONFIRMED PATTERN: Run 8 and Run 16 both use dpo=35mm (largest promoter, tightest annulus, ~15.5mm gap) - this geometry level needs finer local mesh before re-running. Run 27 (also dpo=35mm) is at high risk of the same failure.</t>
   </si>
   <si>
     <t xml:space="preserve">phi1 (=phi2, even-split assumption)</t>
@@ -604,7 +607,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -626,6 +629,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2246,50 +2253,50 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="5" t="n">
         <v>4.55</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="5" t="n">
         <v>0.53</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="5" t="n">
         <v>0.04</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="I18" s="1" t="n">
+      <c r="I18" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="K18" s="1" t="n">
+      <c r="K18" s="5" t="n">
         <v>1.4</v>
       </c>
-      <c r="L18" s="1" t="n">
+      <c r="L18" s="5" t="n">
         <v>32.2</v>
       </c>
-      <c r="M18" s="1" t="n">
+      <c r="M18" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="N18" s="1" t="n">
+      <c r="N18" s="5" t="n">
         <f aca="false">Constants!$C$7</f>
         <v>10000</v>
       </c>
-      <c r="O18" s="1" t="n">
+      <c r="O18" s="5" t="n">
         <f aca="false">Constants!$C$8</f>
         <v>500</v>
       </c>
@@ -3096,14 +3103,27 @@
       <c r="F17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
+      <c r="B18" s="5" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>6054475</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>2334551</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>0.84954</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0.0092812</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
@@ -3246,31 +3266,31 @@
         <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3886,34 +3906,34 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="5" t="n">
         <v>5180</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="5" t="n">
         <v>670</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="5" t="n">
         <v>1800</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="5" t="n">
         <v>717</v>
       </c>
-      <c r="G18" s="1" t="n">
+      <c r="G18" s="5" t="n">
         <v>802.056</v>
       </c>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="5" t="n">
         <v>1850.62</v>
       </c>
-      <c r="I18" s="1" t="n">
+      <c r="I18" s="5" t="n">
         <v>0.102577</v>
       </c>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="5" t="n">
         <v>0.0017911</v>
       </c>
     </row>
@@ -4369,49 +4389,49 @@
         <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4831,24 +4851,24 @@
       <c r="P17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
-      <c r="P18" s="4"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
@@ -5098,52 +5118,52 @@
         <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5199,14 +5219,14 @@
         <v>0.176177681878176</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="O2" s="1" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$O$2/'Fluent Raw Results'!$N$2,"")</f>
         <v/>
       </c>
       <c r="P2" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Q2" s="1" t="n">
         <f aca="false">IFERROR(ABS('Fluent Raw Results'!$B$2-'Fluent Raw Results'!$C$2)/'Fluent Raw Results'!$B$2*100,"")</f>
@@ -6249,70 +6269,70 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="5" t="n">
         <f aca="false">(PI()*Constants!$C$4^2/4-('Run Matrix (Inputs)'!$J$18/1000)^2)+('Run Matrix (Inputs)'!$L$18/1000)^2</f>
         <v>0.00323303439975929</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$18/('Fluid Properties'!$G$18*$B$18),"")</f>
         <v>0</v>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="5" t="n">
         <f aca="false">IFERROR('Fluid Properties'!$G$18*$C$18*Constants!$C$4/'Fluid Properties'!$J$18,"")</f>
         <v>0</v>
       </c>
-      <c r="E18" s="1" t="str">
+      <c r="E18" s="5" t="str">
         <f aca="false">IF(OR('Fluent Raw Results'!$F$18="",'Fluent Raw Results'!$G$18=""),"",('Fluent Raw Results'!$F$18+'Fluent Raw Results'!$G$18)/2)</f>
         <v/>
       </c>
-      <c r="F18" s="1" t="str">
+      <c r="F18" s="5" t="str">
         <f aca="false">IF(OR('Fluent Raw Results'!$D$18="",'Fluent Raw Results'!$E$18=""),"",'Fluent Raw Results'!$D$18-'Fluent Raw Results'!$E$18)</f>
         <v/>
       </c>
-      <c r="G18" s="1" t="str">
+      <c r="G18" s="5" t="str">
         <f aca="false">IFERROR(2*'Fluent Raw Results'!$I$18/('Fluid Properties'!$G$18*$C$18^2),"")</f>
         <v/>
       </c>
-      <c r="H18" s="1" t="str">
+      <c r="H18" s="5" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$J$18/('Fluent Raw Results'!$H$18-$E$18),"")</f>
         <v/>
       </c>
-      <c r="I18" s="1" t="str">
+      <c r="I18" s="5" t="str">
         <f aca="false">IFERROR($H$18*Constants!$C$4/'Fluid Properties'!$I$18,"")</f>
         <v/>
       </c>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$18*'Fluid Properties'!$H$18*('Fluent Raw Results'!$G$18-'Fluent Raw Results'!$F$18),"")</f>
         <v>0</v>
       </c>
-      <c r="K18" s="1" t="str">
+      <c r="K18" s="5" t="str">
         <f aca="false">IFERROR(('Fluent Raw Results'!$B$18/'Fluid Properties'!$G$18)*$F$18,"")</f>
         <v/>
       </c>
-      <c r="L18" s="1" t="str">
+      <c r="L18" s="5" t="str">
         <f aca="false">IFERROR(($J$18-$K$18/Constants!$C$13)/(Constants!$C$9*Constants!$C$10),"")</f>
         <v/>
       </c>
-      <c r="M18" s="1" t="str">
+      <c r="M18" s="5" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$18*'Fluid Properties'!$H$18*(('Fluent Raw Results'!$G$18-'Fluent Raw Results'!$F$18)-Constants!$C$11*LN('Fluent Raw Results'!$G$18/'Fluent Raw Results'!$F$18))/(Constants!$C$9*Constants!$C$10*(1+(1/3)*(Constants!$C$11/Constants!$C$12)^4-(4/3)*(Constants!$C$11/Constants!$C$12))),"")</f>
         <v/>
       </c>
-      <c r="N18" s="1" t="str">
+      <c r="N18" s="5" t="str">
         <f aca="false">IFERROR(($I$18/$I$2)/($G$18/$G$2)^(1/3),"")</f>
         <v/>
       </c>
-      <c r="O18" s="1" t="str">
+      <c r="O18" s="5" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$O$18/'Fluent Raw Results'!$N$18,"")</f>
         <v/>
       </c>
-      <c r="P18" s="1" t="str">
+      <c r="P18" s="5" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$N$18/'Fluent Raw Results'!$N$2,"")</f>
         <v/>
       </c>
-      <c r="Q18" s="1" t="str">
+      <c r="Q18" s="5" t="str">
         <f aca="false">IFERROR(ABS('Fluent Raw Results'!$B$18-'Fluent Raw Results'!$C$18)/'Fluent Raw Results'!$B$18*100,"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add raw diverged Fluent values for Run 8 and Run 16 (kept, red-flagged, not left blank)
</commit_message>
<xml_diff>
--- a/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
+++ b/thesis/production-runs/PTSC_27Run_Master_Workbook.xlsx
@@ -607,7 +607,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -629,10 +629,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3121,7 +3117,7 @@
       <c r="F18" s="5" t="n">
         <v>0.0092812</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="5" t="s">
         <v>118</v>
       </c>
     </row>
@@ -4670,18 +4666,42 @@
       <c r="A10" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+      <c r="B10" s="5" t="n">
+        <v>0.82919118</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>1.5783349E+018</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>2.6597209E+039</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>-8.073603E+033</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>1070.2935</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>907.11549</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>2.6460385E+031</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>35610.373</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>15659.329</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>22522845000000</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>22972189000000000</v>
+      </c>
       <c r="N10" s="5"/>
       <c r="O10" s="5"/>
       <c r="P10" s="5"/>
@@ -4854,18 +4874,42 @@
       <c r="A18" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
+      <c r="B18" s="5" t="n">
+        <v>0.87599111</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>1758631000000000</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>2.7368531E+035</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>-1.2680777E+033</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>4924.9588</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>4.0961628</v>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>35606.134</v>
+      </c>
+      <c r="K18" s="5" t="n">
+        <v>15656.949</v>
+      </c>
+      <c r="L18" s="5" t="n">
+        <v>0.07377021</v>
+      </c>
+      <c r="M18" s="5" t="n">
+        <v>1.1821866</v>
+      </c>
       <c r="N18" s="5"/>
       <c r="O18" s="5"/>
       <c r="P18" s="5"/>
@@ -5726,51 +5770,51 @@
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$10/('Fluid Properties'!$G$10*$B$10),"")</f>
-        <v>0</v>
+        <v>0.33779240348504</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">IFERROR('Fluid Properties'!$G$10*$C$10*Constants!$C$4/'Fluid Properties'!$J$10,"")</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="5" t="str">
+        <v>9983.40460163778</v>
+      </c>
+      <c r="E10" s="5" t="n">
         <f aca="false">IF(OR('Fluent Raw Results'!$F$10="",'Fluent Raw Results'!$G$10=""),"",('Fluent Raw Results'!$F$10+'Fluent Raw Results'!$G$10)/2)</f>
-        <v/>
-      </c>
-      <c r="F10" s="5" t="str">
+        <v>785.14675</v>
+      </c>
+      <c r="F10" s="5" t="n">
         <f aca="false">IF(OR('Fluent Raw Results'!$D$10="",'Fluent Raw Results'!$E$10=""),"",'Fluent Raw Results'!$D$10-'Fluent Raw Results'!$E$10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="5" t="str">
+        <v>2.659728973603E+039</v>
+      </c>
+      <c r="G10" s="5" t="n">
         <f aca="false">IFERROR(2*'Fluent Raw Results'!$I$10/('Fluid Properties'!$G$10*$C$10^2),"")</f>
-        <v/>
-      </c>
-      <c r="H10" s="5" t="str">
+        <v>5.78258073894728E+029</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$J$10/('Fluent Raw Results'!$H$10-$E$10),"")</f>
-        <v/>
-      </c>
-      <c r="I10" s="5" t="str">
+        <v>291.963112843504</v>
+      </c>
+      <c r="I10" s="5" t="n">
         <f aca="false">IFERROR($H$10*Constants!$C$4/'Fluid Properties'!$I$10,"")</f>
-        <v/>
+        <v>187.854640393765</v>
       </c>
       <c r="J10" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$10*'Fluid Properties'!$H$10*('Fluent Raw Results'!$G$10-'Fluent Raw Results'!$F$10),"")</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="5" t="str">
+        <v>875124.097794871</v>
+      </c>
+      <c r="K10" s="5" t="n">
         <f aca="false">IFERROR(('Fluent Raw Results'!$B$10/'Fluid Properties'!$G$10)*$F$10,"")</f>
-        <v/>
-      </c>
-      <c r="L10" s="5" t="str">
+        <v>2.74971299522984E+036</v>
+      </c>
+      <c r="L10" s="5" t="n">
         <f aca="false">IFERROR(($J$10-$K$10/Constants!$C$13)/(Constants!$C$9*Constants!$C$10),"")</f>
-        <v/>
-      </c>
-      <c r="M10" s="5" t="str">
+        <v>-2.33819132247435E+032</v>
+      </c>
+      <c r="M10" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$10*'Fluid Properties'!$H$10*(('Fluent Raw Results'!$G$10-'Fluent Raw Results'!$F$10)-Constants!$C$11*LN('Fluent Raw Results'!$G$10/'Fluent Raw Results'!$F$10))/(Constants!$C$9*Constants!$C$10*(1+(1/3)*(Constants!$C$11/Constants!$C$12)^4-(4/3)*(Constants!$C$11/Constants!$C$12))),"")</f>
-        <v/>
-      </c>
-      <c r="N10" s="5" t="str">
+        <v>14.378236206313</v>
+      </c>
+      <c r="N10" s="5" t="n">
         <f aca="false">IFERROR(($I$10/$I$2)/($G$10/$G$2)^(1/3),"")</f>
-        <v/>
+        <v>2.75379985863795E-011</v>
       </c>
       <c r="O10" s="5" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$O$10/'Fluent Raw Results'!$N$10,"")</f>
@@ -5780,9 +5824,9 @@
         <f aca="false">IFERROR('Fluent Raw Results'!$N$10/'Fluent Raw Results'!$N$2,"")</f>
         <v/>
       </c>
-      <c r="Q10" s="5" t="str">
+      <c r="Q10" s="5" t="n">
         <f aca="false">IFERROR(ABS('Fluent Raw Results'!$B$10-'Fluent Raw Results'!$C$10)/'Fluent Raw Results'!$B$10*100,"")</f>
-        <v/>
+        <v>1.90346320374512E+020</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6278,51 +6322,51 @@
       </c>
       <c r="C18" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$18/('Fluid Properties'!$G$18*$B$18),"")</f>
-        <v>0</v>
+        <v>0.337819473833375</v>
       </c>
       <c r="D18" s="5" t="n">
         <f aca="false">IFERROR('Fluid Properties'!$G$18*$C$18*Constants!$C$4/'Fluid Properties'!$J$18,"")</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="5" t="str">
+        <v>9984.20466178522</v>
+      </c>
+      <c r="E18" s="5" t="n">
         <f aca="false">IF(OR('Fluent Raw Results'!$F$18="",'Fluent Raw Results'!$G$18=""),"",('Fluent Raw Results'!$F$18+'Fluent Raw Results'!$G$18)/2)</f>
-        <v/>
-      </c>
-      <c r="F18" s="5" t="str">
+        <v>400</v>
+      </c>
+      <c r="F18" s="5" t="n">
         <f aca="false">IF(OR('Fluent Raw Results'!$D$18="",'Fluent Raw Results'!$E$18=""),"",'Fluent Raw Results'!$D$18-'Fluent Raw Results'!$E$18)</f>
-        <v/>
-      </c>
-      <c r="G18" s="5" t="str">
+        <v>2.749533877E+035</v>
+      </c>
+      <c r="G18" s="5" t="n">
         <f aca="false">IFERROR(2*'Fluent Raw Results'!$I$18/('Fluid Properties'!$G$18*$C$18^2),"")</f>
-        <v/>
-      </c>
-      <c r="H18" s="5" t="str">
+        <v>0.0895020845661202</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$J$18/('Fluent Raw Results'!$H$18-$E$18),"")</f>
-        <v/>
-      </c>
-      <c r="I18" s="5" t="str">
+        <v>7.86883054051232</v>
+      </c>
+      <c r="I18" s="5" t="n">
         <f aca="false">IFERROR($H$18*Constants!$C$4/'Fluid Properties'!$I$18,"")</f>
-        <v/>
+        <v>5.06295578612957</v>
       </c>
       <c r="J18" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$18*'Fluid Properties'!$H$18*('Fluent Raw Results'!$G$18-'Fluent Raw Results'!$F$18),"")</f>
-        <v>0</v>
-      </c>
-      <c r="K18" s="5" t="str">
+        <v>-324225.33359764</v>
+      </c>
+      <c r="K18" s="5" t="n">
         <f aca="false">IFERROR(('Fluent Raw Results'!$B$18/'Fluid Properties'!$G$18)*$F$18,"")</f>
-        <v/>
-      </c>
-      <c r="L18" s="5" t="str">
+        <v>3.0029913533417E+032</v>
+      </c>
+      <c r="L18" s="5" t="n">
         <f aca="false">IFERROR(($J$18-$K$18/Constants!$C$13)/(Constants!$C$9*Constants!$C$10),"")</f>
-        <v/>
-      </c>
-      <c r="M18" s="5" t="str">
+        <v>-2.55356407597084E+028</v>
+      </c>
+      <c r="M18" s="5" t="n">
         <f aca="false">IFERROR('Fluent Raw Results'!$B$18*'Fluid Properties'!$H$18*(('Fluent Raw Results'!$G$18-'Fluent Raw Results'!$F$18)-Constants!$C$11*LN('Fluent Raw Results'!$G$18/'Fluent Raw Results'!$F$18))/(Constants!$C$9*Constants!$C$10*(1+(1/3)*(Constants!$C$11/Constants!$C$12)^4-(4/3)*(Constants!$C$11/Constants!$C$12))),"")</f>
-        <v/>
-      </c>
-      <c r="N18" s="5" t="str">
+        <v>-2.07666816119953</v>
+      </c>
+      <c r="N18" s="5" t="n">
         <f aca="false">IFERROR(($I$18/$I$2)/($G$18/$G$2)^(1/3),"")</f>
-        <v/>
+        <v>0.0138232691940993</v>
       </c>
       <c r="O18" s="5" t="str">
         <f aca="false">IFERROR('Fluent Raw Results'!$O$18/'Fluent Raw Results'!$N$18,"")</f>
@@ -6332,9 +6376,9 @@
         <f aca="false">IFERROR('Fluent Raw Results'!$N$18/'Fluent Raw Results'!$N$2,"")</f>
         <v/>
       </c>
-      <c r="Q18" s="5" t="str">
+      <c r="Q18" s="5" t="n">
         <f aca="false">IFERROR(ABS('Fluent Raw Results'!$B$18-'Fluent Raw Results'!$C$18)/'Fluent Raw Results'!$B$18*100,"")</f>
-        <v/>
+        <v>2.0075900085333E+017</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>